<commit_message>
fix(tc-api-voucher): xóa HTTP codes + bổ sung output fields BA yêu cầu
- Xóa HTTP status code khỏi Expected Response toàn bộ 93 TC (API trả 200 cho cả failed cases)
- API_01.19: bổ sung applyTypeId, promotionTypeId, policyGroupId vào output data[]
- API_02.25–28: rewrite từ sai spec contents[] sang đúng BA spec discount/applies[]
  (API_02.25: 17 top-level fields; API_02.26: 10 sub-fields applies[])
- API_03.28: bổ sung đủ 17 top-level fields + 10 sub-fields applies[]
- MEMORY.md: cập nhật TC Status cho SC-LIST-006, SC-DETAIL-001/002, SC-APPLY-002/003;
  CLA-VOUCHER-002 resolved (partial); thêm entry TC Generation Log 2026-05-26
- CLAUDE.md: cập nhật trạng thái TC API và clarifications còn lại

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ecom-pdh/03_test-cases/api/AI_ISC_ecom-pdh_v1.1_TC_API_v1.0.xlsx
+++ b/ecom-pdh/03_test-cases/api/AI_ISC_ecom-pdh_v1.1_TC_API_v1.0.xlsx
@@ -111,7 +111,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -133,11 +133,55 @@
         <color rgb="00CCCCCC"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -178,6 +222,8 @@
     <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -565,6 +611,16 @@
           <t>TEST CASE API — Lấy danh sách Voucher</t>
         </is>
       </c>
+      <c r="B1" s="14" t="n"/>
+      <c r="C1" s="14" t="n"/>
+      <c r="D1" s="14" t="n"/>
+      <c r="E1" s="14" t="n"/>
+      <c r="F1" s="14" t="n"/>
+      <c r="G1" s="14" t="n"/>
+      <c r="H1" s="14" t="n"/>
+      <c r="I1" s="14" t="n"/>
+      <c r="J1" s="14" t="n"/>
+      <c r="K1" s="15" t="n"/>
     </row>
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -675,6 +731,16 @@
           <t>Authentication / Authorization</t>
         </is>
       </c>
+      <c r="B6" s="14" t="n"/>
+      <c r="C6" s="14" t="n"/>
+      <c r="D6" s="14" t="n"/>
+      <c r="E6" s="14" t="n"/>
+      <c r="F6" s="14" t="n"/>
+      <c r="G6" s="14" t="n"/>
+      <c r="H6" s="14" t="n"/>
+      <c r="I6" s="14" t="n"/>
+      <c r="J6" s="14" t="n"/>
+      <c r="K6" s="15" t="n"/>
     </row>
     <row r="7" ht="55" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
@@ -709,7 +775,7 @@
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>HTTP 401 — error message: 'Không có quyền truy cập' hoặc tương đương — Không trả dữ liệu voucher</t>
+          <t>error message: 'Không có quyền truy cập' hoặc tương đương — Không trả dữ liệu voucher</t>
         </is>
       </c>
       <c r="H7" s="6" t="inlineStr"/>
@@ -750,7 +816,7 @@
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>HTTP 401 — error message rõ ràng — Không trả dữ liệu voucher</t>
+          <t>error message rõ ràng — Không trả dữ liệu voucher</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr"/>
@@ -791,7 +857,7 @@
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>HTTP 401 — error message: 'Token không hợp lệ' — Không trả dữ liệu voucher</t>
+          <t>error message: 'Token không hợp lệ' — Không trả dữ liệu voucher</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr"/>
@@ -832,7 +898,7 @@
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>HTTP 401 — error message: 'Token đã hết hạn' hoặc tương đương</t>
+          <t>error message: 'Token đã hết hạn' hoặc tương đương</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr"/>
@@ -873,7 +939,7 @@
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>HTTP 401 — error message về format token không hợp lệ</t>
+          <t>error message về format token không hợp lệ</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr"/>
@@ -914,7 +980,7 @@
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>HTTP 401 — signature mismatch — Không trả dữ liệu</t>
+          <t>signature mismatch — Không trả dữ liệu</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr"/>
@@ -955,7 +1021,7 @@
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>HTTP 403 — error message: 'Không có quyền thực hiện thao tác này'</t>
+          <t>error message: 'Không có quyền thực hiện thao tác này'</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr"/>
@@ -996,7 +1062,7 @@
       </c>
       <c r="G14" s="9" t="inlineStr">
         <is>
-          <t>HTTP 400 hoặc 401 — Server từ chối request có duplicate auth header</t>
+          <t>Server từ chối request có duplicate auth header</t>
         </is>
       </c>
       <c r="H14" s="9" t="inlineStr"/>
@@ -1037,7 +1103,7 @@
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>HTTP 400 hoặc 401 — error message: 'Không nhập X-Checkout-Token' — Không hiển thị voucher</t>
+          <t>error message: 'Không nhập X-Checkout-Token' — Không hiển thị voucher</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr"/>
@@ -1078,7 +1144,7 @@
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>HTTP 400 hoặc 401 — error message rõ ràng — Không hiển thị voucher</t>
+          <t>error message rõ ràng — Không hiển thị voucher</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr"/>
@@ -1119,7 +1185,7 @@
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>HTTP 401 — error message: 'Không lấy được voucher' — Không trả dữ liệu</t>
+          <t>error message: 'Không lấy được voucher' — Không trả dữ liệu</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr"/>
@@ -1160,7 +1226,7 @@
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>HTTP 401 — error message: 'Token hết hạn' hoặc tương đương</t>
+          <t>error message: 'Token hết hạn' hoặc tương đương</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr"/>
@@ -1201,7 +1267,7 @@
       </c>
       <c r="G19" s="11" t="inlineStr">
         <is>
-          <t>HTTP 400 — error message format không hợp lệ</t>
+          <t>error message format không hợp lệ</t>
         </is>
       </c>
       <c r="H19" s="11" t="inlineStr"/>
@@ -1242,7 +1308,7 @@
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>HTTP 401 — Không trả dữ liệu — X-Checkout-Token phải hợp lệ để tiếp tục</t>
+          <t>Không trả dữ liệu — X-Checkout-Token phải hợp lệ để tiếp tục</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr"/>
@@ -1283,7 +1349,7 @@
       </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>HTTP 401 — Không trả dữ liệu — cả 2 token phải hợp lệ</t>
+          <t>Không trả dữ liệu — cả 2 token phải hợp lệ</t>
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr"/>
@@ -1324,7 +1390,7 @@
       </c>
       <c r="G22" s="6" t="inlineStr">
         <is>
-          <t>HTTP 401 hoặc 403 — Cross-user token mismatch bị từ chối</t>
+          <t>Cross-user token mismatch bị từ chối</t>
         </is>
       </c>
       <c r="H22" s="6" t="inlineStr"/>
@@ -1365,7 +1431,7 @@
       </c>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>HTTP 401 — Replay attack bị từ chối — token đã invalid</t>
+          <t>Replay attack bị từ chối — token đã invalid</t>
         </is>
       </c>
       <c r="H23" s="6" t="inlineStr"/>
@@ -1406,7 +1472,7 @@
       </c>
       <c r="G24" s="9" t="inlineStr">
         <is>
-          <t>HTTP 401 hoặc 403 — Client-Id mismatch bị từ chối</t>
+          <t>Client-Id mismatch bị từ chối</t>
         </is>
       </c>
       <c r="H24" s="9" t="inlineStr"/>
@@ -1420,6 +1486,16 @@
           <t>Business Flow — Happy Path</t>
         </is>
       </c>
+      <c r="B25" s="14" t="n"/>
+      <c r="C25" s="14" t="n"/>
+      <c r="D25" s="14" t="n"/>
+      <c r="E25" s="14" t="n"/>
+      <c r="F25" s="14" t="n"/>
+      <c r="G25" s="14" t="n"/>
+      <c r="H25" s="14" t="n"/>
+      <c r="I25" s="14" t="n"/>
+      <c r="J25" s="14" t="n"/>
+      <c r="K25" s="15" t="n"/>
     </row>
     <row r="26" ht="55" customHeight="1">
       <c r="A26" s="6" t="inlineStr">
@@ -1454,7 +1530,7 @@
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>HTTP 200 — result=1 — data[] có ít nhất 1 item — Mỗi item có đủ: voucherCode (non-null), voucherType (1 hoặc 2), description, note, expiredDate (dd/MM/yyyy)</t>
+          <t>result=1 — data[] có ít nhất 1 item — Mỗi item có đủ: voucherCode (non-null, string), voucherType (integer, 1 hoặc 2), description (string nếu có), note (string nếu có), expiredDate (format dd/MM/yyyy nếu có), applyTypeId (integer nếu có), promotionTypeId (integer nếu có), policyGroupId (integer nếu có)</t>
         </is>
       </c>
       <c r="H26" s="6" t="inlineStr"/>
@@ -1495,7 +1571,7 @@
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>HTTP 200 — data[] khác với lần gọi trước nếu PTTT/Gói ảnh hưởng đến EVC — Phản ánh đúng context mới</t>
+          <t>data[] khác với lần gọi trước nếu PTTT/Gói ảnh hưởng đến EVC — Phản ánh đúng context mới</t>
         </is>
       </c>
       <c r="H27" s="6" t="inlineStr"/>
@@ -1536,7 +1612,7 @@
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>HTTP 200 — Tất cả voucher trong data[] thuộc đúng kênh hiện tại — Không lẫn voucher kênh khác</t>
+          <t>Tất cả voucher trong data[] thuộc đúng kênh hiện tại — Không lẫn voucher kênh khác</t>
         </is>
       </c>
       <c r="H28" s="6" t="inlineStr"/>
@@ -1550,6 +1626,16 @@
           <t>Business Flow — Edge Cases</t>
         </is>
       </c>
+      <c r="B29" s="14" t="n"/>
+      <c r="C29" s="14" t="n"/>
+      <c r="D29" s="14" t="n"/>
+      <c r="E29" s="14" t="n"/>
+      <c r="F29" s="14" t="n"/>
+      <c r="G29" s="14" t="n"/>
+      <c r="H29" s="14" t="n"/>
+      <c r="I29" s="14" t="n"/>
+      <c r="J29" s="14" t="n"/>
+      <c r="K29" s="15" t="n"/>
     </row>
     <row r="30" ht="55" customHeight="1">
       <c r="A30" s="9" t="inlineStr">
@@ -1584,7 +1670,7 @@
       </c>
       <c r="G30" s="9" t="inlineStr">
         <is>
-          <t>HTTP 200 — result=0 — data[]=[] hoặc null — Không có 4xx/5xx — Không báo lỗi user</t>
+          <t>result=0 — data[]=[] hoặc null — Không có 4xx/5xx — Không báo lỗi user</t>
         </is>
       </c>
       <c r="H30" s="9" t="inlineStr"/>
@@ -1625,7 +1711,7 @@
       </c>
       <c r="G31" s="11" t="inlineStr">
         <is>
-          <t>HTTP 200 — Voucher hết hạn không có trong data[] — Chỉ trả voucher còn hiệu lực</t>
+          <t>Voucher hết hạn không có trong data[] — Chỉ trả voucher còn hiệu lực</t>
         </is>
       </c>
       <c r="H31" s="11" t="inlineStr"/>
@@ -1666,7 +1752,7 @@
       </c>
       <c r="G32" s="9" t="inlineStr">
         <is>
-          <t>HTTP 200 — data[] chứa tất cả voucher hợp lệ — Số lượng item = số voucher hiển thị trên UI</t>
+          <t>data[] chứa tất cả voucher hợp lệ — Số lượng item = số voucher hiển thị trên UI</t>
         </is>
       </c>
       <c r="H32" s="9" t="inlineStr"/>
@@ -1707,7 +1793,7 @@
       </c>
       <c r="G33" s="11" t="inlineStr">
         <is>
-          <t>HTTP 200 — Mỗi item có: voucherCode (non-null), voucherType (integer, 1 hoặc 2) — Không có field null bắt buộc</t>
+          <t>Mỗi item có: voucherCode (non-null), voucherType (integer, 1 hoặc 2) — Không có field null bắt buộc</t>
         </is>
       </c>
       <c r="H33" s="11" t="inlineStr"/>
@@ -1721,6 +1807,16 @@
           <t>Error Handling</t>
         </is>
       </c>
+      <c r="B34" s="14" t="n"/>
+      <c r="C34" s="14" t="n"/>
+      <c r="D34" s="14" t="n"/>
+      <c r="E34" s="14" t="n"/>
+      <c r="F34" s="14" t="n"/>
+      <c r="G34" s="14" t="n"/>
+      <c r="H34" s="14" t="n"/>
+      <c r="I34" s="14" t="n"/>
+      <c r="J34" s="14" t="n"/>
+      <c r="K34" s="15" t="n"/>
     </row>
     <row r="35" ht="55" customHeight="1">
       <c r="A35" s="9" t="inlineStr">
@@ -1755,7 +1851,7 @@
       </c>
       <c r="G35" s="9" t="inlineStr">
         <is>
-          <t>HTTP 404 hoặc 400 — error message rõ ràng — Không crash server</t>
+          <t>error message rõ ràng — Không crash server</t>
         </is>
       </c>
       <c r="H35" s="9" t="inlineStr"/>
@@ -1837,7 +1933,7 @@
       </c>
       <c r="G37" s="9" t="inlineStr">
         <is>
-          <t>HTTP 503 hoặc 504 — error message 'Dịch vụ tạm thời không khả dụng' — Không lộ thông tin nội bộ</t>
+          <t>error message 'Dịch vụ tạm thời không khả dụng' — Không lộ thông tin nội bộ</t>
         </is>
       </c>
       <c r="H37" s="9" t="inlineStr"/>
@@ -1848,8 +1944,8 @@
   </sheetData>
   <mergeCells count="9">
     <mergeCell ref="A6:K6"/>
+    <mergeCell ref="A34:K34"/>
     <mergeCell ref="B3:D3"/>
-    <mergeCell ref="A34:K34"/>
     <mergeCell ref="F3:K3"/>
     <mergeCell ref="A29:K29"/>
     <mergeCell ref="A25:K25"/>
@@ -1889,6 +1985,16 @@
           <t>TEST CASE API — Lấy nội dung chi tiết Voucher</t>
         </is>
       </c>
+      <c r="B1" s="14" t="n"/>
+      <c r="C1" s="14" t="n"/>
+      <c r="D1" s="14" t="n"/>
+      <c r="E1" s="14" t="n"/>
+      <c r="F1" s="14" t="n"/>
+      <c r="G1" s="14" t="n"/>
+      <c r="H1" s="14" t="n"/>
+      <c r="I1" s="14" t="n"/>
+      <c r="J1" s="14" t="n"/>
+      <c r="K1" s="15" t="n"/>
     </row>
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1999,6 +2105,16 @@
           <t>Authentication / Authorization</t>
         </is>
       </c>
+      <c r="B6" s="14" t="n"/>
+      <c r="C6" s="14" t="n"/>
+      <c r="D6" s="14" t="n"/>
+      <c r="E6" s="14" t="n"/>
+      <c r="F6" s="14" t="n"/>
+      <c r="G6" s="14" t="n"/>
+      <c r="H6" s="14" t="n"/>
+      <c r="I6" s="14" t="n"/>
+      <c r="J6" s="14" t="n"/>
+      <c r="K6" s="15" t="n"/>
     </row>
     <row r="7" ht="55" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
@@ -2033,7 +2149,7 @@
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>HTTP 401 — error message: 'Không có quyền truy cập' hoặc tương đương — Không trả dữ liệu voucher</t>
+          <t>error message: 'Không có quyền truy cập' hoặc tương đương — Không trả dữ liệu voucher</t>
         </is>
       </c>
       <c r="H7" s="6" t="inlineStr"/>
@@ -2074,7 +2190,7 @@
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>HTTP 401 — error message rõ ràng — Không trả dữ liệu voucher</t>
+          <t>error message rõ ràng — Không trả dữ liệu voucher</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr"/>
@@ -2115,7 +2231,7 @@
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>HTTP 401 — error message: 'Token không hợp lệ' — Không trả dữ liệu voucher</t>
+          <t>error message: 'Token không hợp lệ' — Không trả dữ liệu voucher</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr"/>
@@ -2156,7 +2272,7 @@
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>HTTP 401 — error message: 'Token đã hết hạn' hoặc tương đương</t>
+          <t>error message: 'Token đã hết hạn' hoặc tương đương</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr"/>
@@ -2197,7 +2313,7 @@
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>HTTP 401 — error message về format token không hợp lệ</t>
+          <t>error message về format token không hợp lệ</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr"/>
@@ -2238,7 +2354,7 @@
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>HTTP 401 — signature mismatch — Không trả dữ liệu</t>
+          <t>signature mismatch — Không trả dữ liệu</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr"/>
@@ -2279,7 +2395,7 @@
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>HTTP 403 — error message: 'Không có quyền thực hiện thao tác này'</t>
+          <t>error message: 'Không có quyền thực hiện thao tác này'</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr"/>
@@ -2320,7 +2436,7 @@
       </c>
       <c r="G14" s="9" t="inlineStr">
         <is>
-          <t>HTTP 400 hoặc 401 — Server từ chối request có duplicate auth header</t>
+          <t>Server từ chối request có duplicate auth header</t>
         </is>
       </c>
       <c r="H14" s="9" t="inlineStr"/>
@@ -2361,7 +2477,7 @@
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>HTTP 400 hoặc 401 — error message: 'Không nhập X-Checkout-Token' — Không hiển thị voucher</t>
+          <t>error message: 'Không nhập X-Checkout-Token' — Không hiển thị voucher</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr"/>
@@ -2402,7 +2518,7 @@
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>HTTP 400 hoặc 401 — error message rõ ràng — Không hiển thị voucher</t>
+          <t>error message rõ ràng — Không hiển thị voucher</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr"/>
@@ -2443,7 +2559,7 @@
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>HTTP 401 — error message: 'Không lấy được voucher' — Không trả dữ liệu</t>
+          <t>error message: 'Không lấy được voucher' — Không trả dữ liệu</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr"/>
@@ -2484,7 +2600,7 @@
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>HTTP 401 — error message: 'Token hết hạn' hoặc tương đương</t>
+          <t>error message: 'Token hết hạn' hoặc tương đương</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr"/>
@@ -2525,7 +2641,7 @@
       </c>
       <c r="G19" s="11" t="inlineStr">
         <is>
-          <t>HTTP 400 — error message format không hợp lệ</t>
+          <t>error message format không hợp lệ</t>
         </is>
       </c>
       <c r="H19" s="11" t="inlineStr"/>
@@ -2566,7 +2682,7 @@
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>HTTP 401 — Không trả dữ liệu — X-Checkout-Token phải hợp lệ để tiếp tục</t>
+          <t>Không trả dữ liệu — X-Checkout-Token phải hợp lệ để tiếp tục</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr"/>
@@ -2607,7 +2723,7 @@
       </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>HTTP 401 — Không trả dữ liệu — cả 2 token phải hợp lệ</t>
+          <t>Không trả dữ liệu — cả 2 token phải hợp lệ</t>
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr"/>
@@ -2648,7 +2764,7 @@
       </c>
       <c r="G22" s="6" t="inlineStr">
         <is>
-          <t>HTTP 401 hoặc 403 — Cross-user token mismatch bị từ chối</t>
+          <t>Cross-user token mismatch bị từ chối</t>
         </is>
       </c>
       <c r="H22" s="6" t="inlineStr"/>
@@ -2689,7 +2805,7 @@
       </c>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>HTTP 401 — Replay attack bị từ chối — token đã invalid</t>
+          <t>Replay attack bị từ chối — token đã invalid</t>
         </is>
       </c>
       <c r="H23" s="6" t="inlineStr"/>
@@ -2730,7 +2846,7 @@
       </c>
       <c r="G24" s="9" t="inlineStr">
         <is>
-          <t>HTTP 401 hoặc 403 — Client-Id mismatch bị từ chối</t>
+          <t>Client-Id mismatch bị từ chối</t>
         </is>
       </c>
       <c r="H24" s="9" t="inlineStr"/>
@@ -2744,6 +2860,16 @@
           <t>Validation — Required Fields</t>
         </is>
       </c>
+      <c r="B25" s="14" t="n"/>
+      <c r="C25" s="14" t="n"/>
+      <c r="D25" s="14" t="n"/>
+      <c r="E25" s="14" t="n"/>
+      <c r="F25" s="14" t="n"/>
+      <c r="G25" s="14" t="n"/>
+      <c r="H25" s="14" t="n"/>
+      <c r="I25" s="14" t="n"/>
+      <c r="J25" s="14" t="n"/>
+      <c r="K25" s="15" t="n"/>
     </row>
     <row r="26" ht="55" customHeight="1">
       <c r="A26" s="6" t="inlineStr">
@@ -2778,7 +2904,7 @@
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>HTTP 400 — error message: 'voucher_code là bắt buộc' — Không gọi QLCS</t>
+          <t>error message: 'voucher_code là bắt buộc' — Không gọi QLCS</t>
         </is>
       </c>
       <c r="H26" s="6" t="inlineStr"/>
@@ -2819,7 +2945,7 @@
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>HTTP 400 — error message về field bắt buộc — Không gọi QLCS</t>
+          <t>error message về field bắt buộc — Không gọi QLCS</t>
         </is>
       </c>
       <c r="H27" s="6" t="inlineStr"/>
@@ -2860,7 +2986,7 @@
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>HTTP 400 — error message về field bắt buộc</t>
+          <t>error message về field bắt buộc</t>
         </is>
       </c>
       <c r="H28" s="6" t="inlineStr"/>
@@ -2874,6 +3000,16 @@
           <t>Validation — Format / Security [SECURITY-INFERRED]</t>
         </is>
       </c>
+      <c r="B29" s="14" t="n"/>
+      <c r="C29" s="14" t="n"/>
+      <c r="D29" s="14" t="n"/>
+      <c r="E29" s="14" t="n"/>
+      <c r="F29" s="14" t="n"/>
+      <c r="G29" s="14" t="n"/>
+      <c r="H29" s="14" t="n"/>
+      <c r="I29" s="14" t="n"/>
+      <c r="J29" s="14" t="n"/>
+      <c r="K29" s="15" t="n"/>
     </row>
     <row r="30" ht="55" customHeight="1">
       <c r="A30" s="9" t="inlineStr">
@@ -2908,7 +3044,7 @@
       </c>
       <c r="G30" s="9" t="inlineStr">
         <is>
-          <t>HTTP 400 — error message về độ dài — Không gọi QLCS — Không crash</t>
+          <t>error message về độ dài — Không gọi QLCS — Không crash</t>
         </is>
       </c>
       <c r="H30" s="9" t="inlineStr"/>
@@ -2949,7 +3085,7 @@
       </c>
       <c r="G31" s="11" t="inlineStr">
         <is>
-          <t>HTTP 400 — Input bị sanitize/reject — Không execute script — Không lộ lỗi nội bộ</t>
+          <t>Input bị sanitize/reject — Không execute script — Không lộ lỗi nội bộ</t>
         </is>
       </c>
       <c r="H31" s="11" t="inlineStr"/>
@@ -2990,7 +3126,7 @@
       </c>
       <c r="G32" s="9" t="inlineStr">
         <is>
-          <t>HTTP 400 — Input bị reject — Không có SQL error trong response — Không lộ cấu trúc DB</t>
+          <t>Input bị reject — Không có SQL error trong response — Không lộ cấu trúc DB</t>
         </is>
       </c>
       <c r="H32" s="9" t="inlineStr"/>
@@ -3004,6 +3140,16 @@
           <t>Business Flow — Happy Path</t>
         </is>
       </c>
+      <c r="B33" s="14" t="n"/>
+      <c r="C33" s="14" t="n"/>
+      <c r="D33" s="14" t="n"/>
+      <c r="E33" s="14" t="n"/>
+      <c r="F33" s="14" t="n"/>
+      <c r="G33" s="14" t="n"/>
+      <c r="H33" s="14" t="n"/>
+      <c r="I33" s="14" t="n"/>
+      <c r="J33" s="14" t="n"/>
+      <c r="K33" s="15" t="n"/>
     </row>
     <row r="34" ht="55" customHeight="1">
       <c r="A34" s="6" t="inlineStr">
@@ -3023,22 +3169,22 @@
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
-          <t>Lấy nội dung voucher thành công — QLCS có content</t>
+          <t>Lấy nội dung voucher thành công — validate top-level output fields theo BA spec</t>
         </is>
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>Checkout hợp lệ; Authorization + X-Checkout-Token hợp lệ; voucherCode lấy từ API list; QLCS có nội dung cho voucher này</t>
+          <t>Checkout hợp lệ; Authorization + X-Checkout-Token hợp lệ; voucher_code lấy từ API list; QLCS trả đầy đủ thông tin voucher</t>
         </is>
       </c>
       <c r="F34" s="6" t="inlineStr">
         <is>
-          <t>POST /public/v1/voucher/content với voucher_code hợp lệ</t>
+          <t>POST /public/v1/voucher/content với voucher_code hợp lệ; kiểm tra response body</t>
         </is>
       </c>
       <c r="G34" s="6" t="inlineStr">
         <is>
-          <t>HTTP 200 — success=true — voucherCode khớp input — contents[] có ít nhất 1 phần tử không rỗng</t>
+          <t>success=true — voucher_code khớp input (non-null, string) — voucher_type là integer cấp 1 (non-null) — Response có đủ: promotion_id (string), promotion_title (string), referrer_code, discount_type (string), discount_value (number ≥ 0), discount_ex_vat_value (number), discount_rate (number), apply_type, apply_from, apply_to, original_discount_value (number), original_discount_ex_vat (number), voucher_type_l2 (integer), type_id (integer)</t>
         </is>
       </c>
       <c r="H34" s="6" t="inlineStr"/>
@@ -3064,22 +3210,22 @@
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>contents[] lọc đúng Content rỗng và null từ QLCS</t>
+          <t>Validate applies[] sub-fields đủ và đúng kiểu dữ liệu</t>
         </is>
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>QLCS trả Content3='', Content4=null cho voucher này</t>
+          <t>QLCS trả applies[] có ít nhất 1 item; voucher có áp chiết khấu dịch vụ</t>
         </is>
       </c>
       <c r="F35" s="6" t="inlineStr">
         <is>
-          <t>POST /public/v1/voucher/content</t>
+          <t>POST /public/v1/voucher/content; kiểm tra schema applies[] trong response</t>
         </is>
       </c>
       <c r="G35" s="6" t="inlineStr">
         <is>
-          <t>HTTP 200 — contents[] KHÔNG chứa chuỗi rỗng hoặc null — Chỉ giữ lại phần tử có giá trị thực</t>
+          <t>applies[] có ít nhất 1 item — Mỗi item có đủ: service_id (integer), sub_service_type_id (integer), sub_service_id (integer), service_code (integer), discount_ex_vat (number), discount (number), dismonth (integer; 0 = áp 1 lần), is_deduct_order (integer; 1 = khấu trừ trực tiếp vào tổng đơn), original_discount_value (number), original_discount_ex_vat (number)</t>
         </is>
       </c>
       <c r="H35" s="6" t="inlineStr"/>
@@ -3105,22 +3251,22 @@
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
-          <t>Thứ tự contents[] đúng: Content1 trước Content6</t>
+          <t>Validate required fields non-null: voucher_code và voucher_type luôn có giá trị</t>
         </is>
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>QLCS trả Content1, Content3, Content5 (Content2,4,6 rỗng)</t>
+          <t>QLCS trả data đầy đủ cho voucher hợp lệ</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>POST /public/v1/voucher/content</t>
+          <t>POST /public/v1/voucher/content; kiểm tra required fields trong response</t>
         </is>
       </c>
       <c r="G36" s="6" t="inlineStr">
         <is>
-          <t>HTTP 200 — contents[] = [Content1, Content3, Content5] — Đúng thứ tự, không lộn</t>
+          <t>voucher_code không null, không rỗng (string) — voucher_type không null (integer, cấp 1) — Không có field required nào trả về null trong response thành công</t>
         </is>
       </c>
       <c r="H36" s="6" t="inlineStr"/>
@@ -3134,6 +3280,16 @@
           <t>Business Flow — Edge Cases</t>
         </is>
       </c>
+      <c r="B37" s="14" t="n"/>
+      <c r="C37" s="14" t="n"/>
+      <c r="D37" s="14" t="n"/>
+      <c r="E37" s="14" t="n"/>
+      <c r="F37" s="14" t="n"/>
+      <c r="G37" s="14" t="n"/>
+      <c r="H37" s="14" t="n"/>
+      <c r="I37" s="14" t="n"/>
+      <c r="J37" s="14" t="n"/>
+      <c r="K37" s="15" t="n"/>
     </row>
     <row r="38" ht="55" customHeight="1">
       <c r="A38" s="9" t="inlineStr">
@@ -3153,22 +3309,22 @@
       </c>
       <c r="D38" s="9" t="inlineStr">
         <is>
-          <t>Voucher có tất cả Content fields rỗng → contents[] = []</t>
+          <t>Validate numeric fields đúng kiểu: discount_value, discount_ex_vat_value ≥ 0</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
         <is>
-          <t>QLCS trả tất cả Content1–Content6 đều rỗng</t>
+          <t>QLCS trả đủ discount fields; voucher có giảm giá</t>
         </is>
       </c>
       <c r="F38" s="9" t="inlineStr">
         <is>
-          <t>POST /public/v1/voucher/content</t>
+          <t>POST /public/v1/voucher/content; kiểm tra kiểu dữ liệu và giá trị numeric fields</t>
         </is>
       </c>
       <c r="G38" s="9" t="inlineStr">
         <is>
-          <t>HTTP 200 — success=true — contents=[] — FE hiển thị 'Không có thông tin điều kiện'</t>
+          <t>discount_value là number ≥ 0, không phải string — discount_ex_vat_value là number ≥ 0 — discount_rate là number (0–100 nếu có) — original_discount_value, original_discount_ex_vat là number — Không có giá trị âm không hợp lệ</t>
         </is>
       </c>
       <c r="H38" s="9" t="inlineStr"/>
@@ -3250,7 +3406,7 @@
       </c>
       <c r="G40" s="6" t="inlineStr">
         <is>
-          <t>HTTP 200 — success=false — errorMessage tiếng Việt — Không chứa tên API/field QLCS — Popup list vẫn giữ nguyên</t>
+          <t>success=false — errorMessage tiếng Việt — Không chứa tên API/field QLCS — Popup list vẫn giữ nguyên</t>
         </is>
       </c>
       <c r="H40" s="6" t="inlineStr"/>
@@ -3305,6 +3461,16 @@
           <t>Error Handling</t>
         </is>
       </c>
+      <c r="B42" s="14" t="n"/>
+      <c r="C42" s="14" t="n"/>
+      <c r="D42" s="14" t="n"/>
+      <c r="E42" s="14" t="n"/>
+      <c r="F42" s="14" t="n"/>
+      <c r="G42" s="14" t="n"/>
+      <c r="H42" s="14" t="n"/>
+      <c r="I42" s="14" t="n"/>
+      <c r="J42" s="14" t="n"/>
+      <c r="K42" s="15" t="n"/>
     </row>
     <row r="43" ht="55" customHeight="1">
       <c r="A43" s="9" t="inlineStr">
@@ -3339,7 +3505,7 @@
       </c>
       <c r="G43" s="9" t="inlineStr">
         <is>
-          <t>HTTP 503 hoặc 504 — error message 'Không lấy được thông tin voucher' — Không crash — Không lộ stack trace</t>
+          <t>error message 'Không lấy được thông tin voucher' — Không crash — Không lộ stack trace</t>
         </is>
       </c>
       <c r="H43" s="9" t="inlineStr"/>
@@ -3393,6 +3559,16 @@
           <t>TEST CASE API — Áp dụng / Hủy Voucher</t>
         </is>
       </c>
+      <c r="B1" s="14" t="n"/>
+      <c r="C1" s="14" t="n"/>
+      <c r="D1" s="14" t="n"/>
+      <c r="E1" s="14" t="n"/>
+      <c r="F1" s="14" t="n"/>
+      <c r="G1" s="14" t="n"/>
+      <c r="H1" s="14" t="n"/>
+      <c r="I1" s="14" t="n"/>
+      <c r="J1" s="14" t="n"/>
+      <c r="K1" s="15" t="n"/>
     </row>
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -3503,6 +3679,16 @@
           <t>Authentication / Authorization</t>
         </is>
       </c>
+      <c r="B6" s="14" t="n"/>
+      <c r="C6" s="14" t="n"/>
+      <c r="D6" s="14" t="n"/>
+      <c r="E6" s="14" t="n"/>
+      <c r="F6" s="14" t="n"/>
+      <c r="G6" s="14" t="n"/>
+      <c r="H6" s="14" t="n"/>
+      <c r="I6" s="14" t="n"/>
+      <c r="J6" s="14" t="n"/>
+      <c r="K6" s="15" t="n"/>
     </row>
     <row r="7" ht="55" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
@@ -3537,7 +3723,7 @@
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>HTTP 401 — error message: 'Không có quyền truy cập' hoặc tương đương — Không trả dữ liệu voucher</t>
+          <t>error message: 'Không có quyền truy cập' hoặc tương đương — Không trả dữ liệu voucher</t>
         </is>
       </c>
       <c r="H7" s="6" t="inlineStr"/>
@@ -3578,7 +3764,7 @@
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>HTTP 401 — error message rõ ràng — Không trả dữ liệu voucher</t>
+          <t>error message rõ ràng — Không trả dữ liệu voucher</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr"/>
@@ -3619,7 +3805,7 @@
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>HTTP 401 — error message: 'Token không hợp lệ' — Không trả dữ liệu voucher</t>
+          <t>error message: 'Token không hợp lệ' — Không trả dữ liệu voucher</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr"/>
@@ -3660,7 +3846,7 @@
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>HTTP 401 — error message: 'Token đã hết hạn' hoặc tương đương</t>
+          <t>error message: 'Token đã hết hạn' hoặc tương đương</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr"/>
@@ -3701,7 +3887,7 @@
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>HTTP 401 — error message về format token không hợp lệ</t>
+          <t>error message về format token không hợp lệ</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr"/>
@@ -3742,7 +3928,7 @@
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>HTTP 401 — signature mismatch — Không trả dữ liệu</t>
+          <t>signature mismatch — Không trả dữ liệu</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr"/>
@@ -3783,7 +3969,7 @@
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>HTTP 403 — error message: 'Không có quyền thực hiện thao tác này'</t>
+          <t>error message: 'Không có quyền thực hiện thao tác này'</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr"/>
@@ -3824,7 +4010,7 @@
       </c>
       <c r="G14" s="9" t="inlineStr">
         <is>
-          <t>HTTP 400 hoặc 401 — Server từ chối request có duplicate auth header</t>
+          <t>Server từ chối request có duplicate auth header</t>
         </is>
       </c>
       <c r="H14" s="9" t="inlineStr"/>
@@ -3865,7 +4051,7 @@
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>HTTP 400 hoặc 401 — error message: 'Không nhập X-Checkout-Token' — Không hiển thị voucher</t>
+          <t>error message: 'Không nhập X-Checkout-Token' — Không hiển thị voucher</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr"/>
@@ -3906,7 +4092,7 @@
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>HTTP 400 hoặc 401 — error message rõ ràng — Không hiển thị voucher</t>
+          <t>error message rõ ràng — Không hiển thị voucher</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr"/>
@@ -3947,7 +4133,7 @@
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>HTTP 401 — error message: 'Không lấy được voucher' — Không trả dữ liệu</t>
+          <t>error message: 'Không lấy được voucher' — Không trả dữ liệu</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr"/>
@@ -3988,7 +4174,7 @@
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>HTTP 401 — error message: 'Token hết hạn' hoặc tương đương</t>
+          <t>error message: 'Token hết hạn' hoặc tương đương</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr"/>
@@ -4029,7 +4215,7 @@
       </c>
       <c r="G19" s="11" t="inlineStr">
         <is>
-          <t>HTTP 400 — error message format không hợp lệ</t>
+          <t>error message format không hợp lệ</t>
         </is>
       </c>
       <c r="H19" s="11" t="inlineStr"/>
@@ -4070,7 +4256,7 @@
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>HTTP 401 — Không trả dữ liệu — X-Checkout-Token phải hợp lệ để tiếp tục</t>
+          <t>Không trả dữ liệu — X-Checkout-Token phải hợp lệ để tiếp tục</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr"/>
@@ -4111,7 +4297,7 @@
       </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>HTTP 401 — Không trả dữ liệu — cả 2 token phải hợp lệ</t>
+          <t>Không trả dữ liệu — cả 2 token phải hợp lệ</t>
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr"/>
@@ -4152,7 +4338,7 @@
       </c>
       <c r="G22" s="6" t="inlineStr">
         <is>
-          <t>HTTP 401 hoặc 403 — Cross-user token mismatch bị từ chối</t>
+          <t>Cross-user token mismatch bị từ chối</t>
         </is>
       </c>
       <c r="H22" s="6" t="inlineStr"/>
@@ -4193,7 +4379,7 @@
       </c>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>HTTP 401 — Replay attack bị từ chối — token đã invalid</t>
+          <t>Replay attack bị từ chối — token đã invalid</t>
         </is>
       </c>
       <c r="H23" s="6" t="inlineStr"/>
@@ -4234,7 +4420,7 @@
       </c>
       <c r="G24" s="9" t="inlineStr">
         <is>
-          <t>HTTP 401 hoặc 403 — Client-Id mismatch bị từ chối</t>
+          <t>Client-Id mismatch bị từ chối</t>
         </is>
       </c>
       <c r="H24" s="9" t="inlineStr"/>
@@ -4248,6 +4434,16 @@
           <t>Validation — Required Fields</t>
         </is>
       </c>
+      <c r="B25" s="14" t="n"/>
+      <c r="C25" s="14" t="n"/>
+      <c r="D25" s="14" t="n"/>
+      <c r="E25" s="14" t="n"/>
+      <c r="F25" s="14" t="n"/>
+      <c r="G25" s="14" t="n"/>
+      <c r="H25" s="14" t="n"/>
+      <c r="I25" s="14" t="n"/>
+      <c r="J25" s="14" t="n"/>
+      <c r="K25" s="15" t="n"/>
     </row>
     <row r="26" ht="55" customHeight="1">
       <c r="A26" s="6" t="inlineStr">
@@ -4282,7 +4478,7 @@
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>HTTP 400 — error message: 'vouchers là bắt buộc' — Checkout không thay đổi</t>
+          <t>error message: 'vouchers là bắt buộc' — Checkout không thay đổi</t>
         </is>
       </c>
       <c r="H26" s="6" t="inlineStr"/>
@@ -4323,7 +4519,7 @@
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>HTTP 400 — error message về field bắt buộc — Checkout không thay đổi</t>
+          <t>error message về field bắt buộc — Checkout không thay đổi</t>
         </is>
       </c>
       <c r="H27" s="6" t="inlineStr"/>
@@ -4364,7 +4560,7 @@
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>HTTP 400 — error message: 'voucher_code là bắt buộc' — Không gọi QLCS</t>
+          <t>error message: 'voucher_code là bắt buộc' — Không gọi QLCS</t>
         </is>
       </c>
       <c r="H28" s="6" t="inlineStr"/>
@@ -4405,7 +4601,7 @@
       </c>
       <c r="G29" s="6" t="inlineStr">
         <is>
-          <t>HTTP 400 — error message: 'voucher_type là bắt buộc' — Không gọi QLCS</t>
+          <t>error message: 'voucher_type là bắt buộc' — Không gọi QLCS</t>
         </is>
       </c>
       <c r="H29" s="6" t="inlineStr"/>
@@ -4446,7 +4642,7 @@
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
-          <t>HTTP 400 — error message về field rỗng — Không gọi QLCS</t>
+          <t>error message về field rỗng — Không gọi QLCS</t>
         </is>
       </c>
       <c r="H30" s="6" t="inlineStr"/>
@@ -4487,7 +4683,7 @@
       </c>
       <c r="G31" s="9" t="inlineStr">
         <is>
-          <t>HTTP 400 — error message về giá trị voucher_type không hợp lệ</t>
+          <t>error message về giá trị voucher_type không hợp lệ</t>
         </is>
       </c>
       <c r="H31" s="9" t="inlineStr"/>
@@ -4501,6 +4697,16 @@
           <t>Validation — Security [SECURITY-INFERRED]</t>
         </is>
       </c>
+      <c r="B32" s="14" t="n"/>
+      <c r="C32" s="14" t="n"/>
+      <c r="D32" s="14" t="n"/>
+      <c r="E32" s="14" t="n"/>
+      <c r="F32" s="14" t="n"/>
+      <c r="G32" s="14" t="n"/>
+      <c r="H32" s="14" t="n"/>
+      <c r="I32" s="14" t="n"/>
+      <c r="J32" s="14" t="n"/>
+      <c r="K32" s="15" t="n"/>
     </row>
     <row r="33" ht="55" customHeight="1">
       <c r="A33" s="11" t="inlineStr">
@@ -4535,7 +4741,7 @@
       </c>
       <c r="G33" s="11" t="inlineStr">
         <is>
-          <t>HTTP 400 — error message: 'Trùng lặp voucher_code' — Không cho apply 2 lần cùng 1 voucher</t>
+          <t>error message: 'Trùng lặp voucher_code' — Không cho apply 2 lần cùng 1 voucher</t>
         </is>
       </c>
       <c r="H33" s="11" t="inlineStr"/>
@@ -4576,7 +4782,7 @@
       </c>
       <c r="G34" s="9" t="inlineStr">
         <is>
-          <t>HTTP 400 hoặc 422 — QLCS hoặc CO từ chối — error message rõ ràng về voucher đã dùng</t>
+          <t>QLCS hoặc CO từ chối — error message rõ ràng về voucher đã dùng</t>
         </is>
       </c>
       <c r="H34" s="9" t="inlineStr"/>
@@ -4590,6 +4796,16 @@
           <t>Business Flow — Áp dụng Voucher lần đầu (UC-04.a)</t>
         </is>
       </c>
+      <c r="B35" s="14" t="n"/>
+      <c r="C35" s="14" t="n"/>
+      <c r="D35" s="14" t="n"/>
+      <c r="E35" s="14" t="n"/>
+      <c r="F35" s="14" t="n"/>
+      <c r="G35" s="14" t="n"/>
+      <c r="H35" s="14" t="n"/>
+      <c r="I35" s="14" t="n"/>
+      <c r="J35" s="14" t="n"/>
+      <c r="K35" s="15" t="n"/>
     </row>
     <row r="36" ht="55" customHeight="1">
       <c r="A36" s="6" t="inlineStr">
@@ -4624,7 +4840,7 @@
       </c>
       <c r="G36" s="6" t="inlineStr">
         <is>
-          <t>HTTP 200 — success=true — appliedVoucher.voucherCode = 'CA21060100KTHIETBIKHOFG039' — discountLines[].discountAmount &gt; 0 — newOrderTotal = giá gốc - tổng discount</t>
+          <t>success=true — appliedVoucher.voucherCode = 'CA21060100KTHIETBIKHOFG039' — discountLines[].discountAmount &gt; 0 — newOrderTotal = giá gốc - tổng discount</t>
         </is>
       </c>
       <c r="H36" s="6" t="inlineStr"/>
@@ -4665,7 +4881,7 @@
       </c>
       <c r="G37" s="6" t="inlineStr">
         <is>
-          <t>HTTP 200 — success=true — Response chứa: promotion_id, promotion_title, voucher_code, discount_value, applies[] (service_id, discount, dismonth, is_deduct_order)</t>
+          <t>success=true — Response chứa đủ top-level fields: promotion_id (string), promotion_title (string), voucher_code (non-null, string), referrer_code, discount_type (string), discount_value (number ≥ 0), discount_ex_vat_value (number), discount_rate (number), apply_type, apply_from, apply_to, original_discount_value (number), original_discount_ex_vat (number), voucher_type (integer, non-null, cấp 1), voucher_type_l2 (integer), type_id (integer) — applies[] có ít nhất 1 item với đủ sub-fields: service_id (integer), sub_service_type_id (integer), sub_service_id (integer), service_code (integer), discount_ex_vat (number), discount (number), dismonth (integer; 0=áp 1 lần), is_deduct_order (integer; 1=khấu trừ trực tiếp), original_discount_value (number), original_discount_ex_vat (number)</t>
         </is>
       </c>
       <c r="H37" s="6" t="inlineStr"/>
@@ -4706,7 +4922,7 @@
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
-          <t>HTTP 200 — success=false — errorMessage tiếng Việt, không lộ cấu trúc QLCS — Model checkout không thay đổi (Promotion vẫn như cũ)</t>
+          <t>success=false — errorMessage tiếng Việt, không lộ cấu trúc QLCS — Model checkout không thay đổi (Promotion vẫn như cũ)</t>
         </is>
       </c>
       <c r="H38" s="6" t="inlineStr"/>
@@ -4720,6 +4936,16 @@
           <t>Business Flow — Apply thêm voucher (UC-04.b)</t>
         </is>
       </c>
+      <c r="B39" s="14" t="n"/>
+      <c r="C39" s="14" t="n"/>
+      <c r="D39" s="14" t="n"/>
+      <c r="E39" s="14" t="n"/>
+      <c r="F39" s="14" t="n"/>
+      <c r="G39" s="14" t="n"/>
+      <c r="H39" s="14" t="n"/>
+      <c r="I39" s="14" t="n"/>
+      <c r="J39" s="14" t="n"/>
+      <c r="K39" s="15" t="n"/>
     </row>
     <row r="40" ht="55" customHeight="1">
       <c r="A40" s="6" t="inlineStr">
@@ -4754,7 +4980,7 @@
       </c>
       <c r="G40" s="6" t="inlineStr">
         <is>
-          <t>HTTP 200 — success=true — Cả voucher A và B được apply — discountLines phản ánh cả 2 voucher — newOrderTotal giảm theo cả 2</t>
+          <t>success=true — Cả voucher A và B được apply — discountLines phản ánh cả 2 voucher — newOrderTotal giảm theo cả 2</t>
         </is>
       </c>
       <c r="H40" s="6" t="inlineStr"/>
@@ -4795,7 +5021,7 @@
       </c>
       <c r="G41" s="6" t="inlineStr">
         <is>
-          <t>HTTP 200 — success=false (cho B) — appliedVoucher vẫn là voucher A — newOrderTotal vẫn = giá sau giảm A — Voucher A không bị xóa</t>
+          <t>success=false (cho B) — appliedVoucher vẫn là voucher A — newOrderTotal vẫn = giá sau giảm A — Voucher A không bị xóa</t>
         </is>
       </c>
       <c r="H41" s="6" t="inlineStr"/>
@@ -4836,7 +5062,7 @@
       </c>
       <c r="G42" s="9" t="inlineStr">
         <is>
-          <t>HTTP 200 — success=false — errorMessage tiếng Việt — Checkout không thay đổi</t>
+          <t>success=false — errorMessage tiếng Việt — Checkout không thay đổi</t>
         </is>
       </c>
       <c r="H42" s="9" t="inlineStr"/>
@@ -4850,6 +5076,16 @@
           <t>Business Flow — Hủy Voucher (UC-05)</t>
         </is>
       </c>
+      <c r="B43" s="14" t="n"/>
+      <c r="C43" s="14" t="n"/>
+      <c r="D43" s="14" t="n"/>
+      <c r="E43" s="14" t="n"/>
+      <c r="F43" s="14" t="n"/>
+      <c r="G43" s="14" t="n"/>
+      <c r="H43" s="14" t="n"/>
+      <c r="I43" s="14" t="n"/>
+      <c r="J43" s="14" t="n"/>
+      <c r="K43" s="15" t="n"/>
     </row>
     <row r="44" ht="55" customHeight="1">
       <c r="A44" s="6" t="inlineStr">
@@ -4884,7 +5120,7 @@
       </c>
       <c r="G44" s="6" t="inlineStr">
         <is>
-          <t>HTTP 200 — success=true — Promotion=[] trong model checkout — DiscountAllocation=0 — newOrderTotal = giá gốc trước UC-04 — CO không gọi QLCS (xử lý nội bộ)</t>
+          <t>success=true — Promotion=[] trong model checkout — DiscountAllocation=0 — newOrderTotal = giá gốc trước UC-04 — CO không gọi QLCS (xử lý nội bộ)</t>
         </is>
       </c>
       <c r="H44" s="6" t="inlineStr"/>
@@ -4925,7 +5161,7 @@
       </c>
       <c r="G45" s="6" t="inlineStr">
         <is>
-          <t>HTTP 200 — newOrderTotal trong response == GT (giá gốc ban đầu) — Không có sai lệch số học</t>
+          <t>newOrderTotal trong response == GT (giá gốc ban đầu) — Không có sai lệch số học</t>
         </is>
       </c>
       <c r="H45" s="6" t="inlineStr"/>
@@ -5021,6 +5257,16 @@
           <t>Business Flow — Recheck khi hoàn tất checkout (UC-06)</t>
         </is>
       </c>
+      <c r="B48" s="14" t="n"/>
+      <c r="C48" s="14" t="n"/>
+      <c r="D48" s="14" t="n"/>
+      <c r="E48" s="14" t="n"/>
+      <c r="F48" s="14" t="n"/>
+      <c r="G48" s="14" t="n"/>
+      <c r="H48" s="14" t="n"/>
+      <c r="I48" s="14" t="n"/>
+      <c r="J48" s="14" t="n"/>
+      <c r="K48" s="15" t="n"/>
     </row>
     <row r="49" ht="55" customHeight="1">
       <c r="A49" s="6" t="inlineStr">
@@ -5151,6 +5397,16 @@
           <t>Business Flow — Auto Apply (UC-01, UC-02)</t>
         </is>
       </c>
+      <c r="B52" s="14" t="n"/>
+      <c r="C52" s="14" t="n"/>
+      <c r="D52" s="14" t="n"/>
+      <c r="E52" s="14" t="n"/>
+      <c r="F52" s="14" t="n"/>
+      <c r="G52" s="14" t="n"/>
+      <c r="H52" s="14" t="n"/>
+      <c r="I52" s="14" t="n"/>
+      <c r="J52" s="14" t="n"/>
+      <c r="K52" s="15" t="n"/>
     </row>
     <row r="53" ht="55" customHeight="1">
       <c r="A53" s="6" t="inlineStr">
@@ -5486,6 +5742,16 @@
           <t>Error Handling</t>
         </is>
       </c>
+      <c r="B61" s="14" t="n"/>
+      <c r="C61" s="14" t="n"/>
+      <c r="D61" s="14" t="n"/>
+      <c r="E61" s="14" t="n"/>
+      <c r="F61" s="14" t="n"/>
+      <c r="G61" s="14" t="n"/>
+      <c r="H61" s="14" t="n"/>
+      <c r="I61" s="14" t="n"/>
+      <c r="J61" s="14" t="n"/>
+      <c r="K61" s="15" t="n"/>
     </row>
     <row r="62" ht="55" customHeight="1">
       <c r="A62" s="9" t="inlineStr">
@@ -5520,7 +5786,7 @@
       </c>
       <c r="G62" s="9" t="inlineStr">
         <is>
-          <t>HTTP 503 hoặc 504 — error message 'Dịch vụ tạm thời không khả dụng' — Checkout không thay đổi — Không lộ thông tin nội bộ</t>
+          <t>error message 'Dịch vụ tạm thời không khả dụng' — Checkout không thay đổi — Không lộ thông tin nội bộ</t>
         </is>
       </c>
       <c r="H62" s="9" t="inlineStr"/>
@@ -5561,7 +5827,7 @@
       </c>
       <c r="G63" s="11" t="inlineStr">
         <is>
-          <t>HTTP 404 hoặc 400 — error message rõ ràng — Không crash server</t>
+          <t>error message rõ ràng — Không crash server</t>
         </is>
       </c>
       <c r="H63" s="11" t="inlineStr"/>

</xml_diff>